<commit_message>
Add erosion validation CSV; update notebook
Add a new erosion_threshold_validation.csv containing monthly validation metrics and pass/score fields. Update research.ipynb to clean outputs, bump execution counts, switch pip shell commands to %pip, add %pip install openpyxl, and reorganize imports (including sklearn utilities and statsmodels plotting helpers); also remove large inline HTML outputs to reduce notebook noise. Binary research-dataset/events.xlsx was updated (file changed). These changes make the notebook more portable and add a dedicated CSV for threshold validation.
</commit_message>
<xml_diff>
--- a/research-dataset/events.xlsx
+++ b/research-dataset/events.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thima\Downloads\data\event labels\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thima\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5391DAD8-2A69-4277-BFDD-F3B2F6D58281}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D67D05BE-5E2C-4C4B-B2B8-F37F40AB163E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="19">
   <si>
     <t>Period</t>
   </si>
@@ -82,9 +82,6 @@
   </si>
   <si>
     <t>Label</t>
-  </si>
-  <si>
-    <t>stable</t>
   </si>
 </sst>
 </file>
@@ -428,7 +425,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
@@ -436,7 +433,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
@@ -452,7 +449,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
@@ -468,7 +465,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
@@ -476,7 +473,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
@@ -484,7 +481,7 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
@@ -492,7 +489,7 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
@@ -500,7 +497,7 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
@@ -508,7 +505,7 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
@@ -532,7 +529,7 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">

</xml_diff>